<commit_message>
Moves mobile industrial equipment to "other processes" element; incorporates new structure for cost allocation thereof; updates shareweights
</commit_message>
<xml_diff>
--- a/InputData/indst/IECCpUAEU/Indst Eqpt Cap Cost per Unit Ann E Use.xlsx
+++ b/InputData/indst/IECCpUAEU/Indst Eqpt Cap Cost per Unit Ann E Use.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\indst\IECCpUAEU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\IECCpUAEU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDBC3E67-205D-4B5E-A078-77723FE107F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D8BEB0-1EC6-4DE8-91A8-15757244A839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30135" yWindow="960" windowWidth="21600" windowHeight="11175" firstSheet="3" activeTab="8" xr2:uid="{6A73F6BA-E2AF-4EFC-B7D0-AD586970A910}"/>
+    <workbookView xWindow="-28410" yWindow="390" windowWidth="22785" windowHeight="14010" tabRatio="762" firstSheet="3" activeTab="10" xr2:uid="{6A73F6BA-E2AF-4EFC-B7D0-AD586970A910}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,9 @@
     <sheet name="Machine Drive" sheetId="5" r:id="rId6"/>
     <sheet name="Electrochemical" sheetId="6" r:id="rId7"/>
     <sheet name="Other" sheetId="10" r:id="rId8"/>
-    <sheet name="IECCpUAEU" sheetId="2" r:id="rId9"/>
+    <sheet name="Other (mobile)" sheetId="11" r:id="rId9"/>
+    <sheet name="IECCpUAEU" sheetId="2" r:id="rId10"/>
+    <sheet name="IECCpUAEU-mobile" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="450">
   <si>
     <t>Sources:</t>
   </si>
@@ -1294,16 +1296,158 @@
   <si>
     <t>low carbon hydrogen if</t>
   </si>
+  <si>
+    <t>Diesel</t>
+  </si>
+  <si>
+    <t>Ag tractors</t>
+  </si>
+  <si>
+    <t>from https://environmentaldevices.com/wp-content/uploads/2023/09/Impacts-of-electrifying-agricultural-tractors.pdf</t>
+  </si>
+  <si>
+    <t>DT #1</t>
+  </si>
+  <si>
+    <t>DT #2</t>
+  </si>
+  <si>
+    <t>DT #3</t>
+  </si>
+  <si>
+    <t>Capital costs</t>
+  </si>
+  <si>
+    <t>eT</t>
+  </si>
+  <si>
+    <t>Tank capacity (gal)</t>
+  </si>
+  <si>
+    <t>Battery capacity (kWh)</t>
+  </si>
+  <si>
+    <t>Runtime/tank (hr)</t>
+  </si>
+  <si>
+    <t>Energy content/tank</t>
+  </si>
+  <si>
+    <t>Energy content:</t>
+  </si>
+  <si>
+    <t>BTU/gal diesel</t>
+  </si>
+  <si>
+    <t>https://afdc.energy.gov/fuels/properties</t>
+  </si>
+  <si>
+    <t>E Intensity (BTU/hr)</t>
+  </si>
+  <si>
+    <t>from https://www.cadeogroup.com/wp-content/uploads/2022/04/PNW-Tractor-Electrification-Study.pdf</t>
+  </si>
+  <si>
+    <t>Energy reservoir (kWh)</t>
+  </si>
+  <si>
+    <t>diesel</t>
+  </si>
+  <si>
+    <t>battery</t>
+  </si>
+  <si>
+    <t>from https://pub.epsilon.slu.se/id/document/20368600</t>
+  </si>
+  <si>
+    <t>example 1</t>
+  </si>
+  <si>
+    <t>example 2</t>
+  </si>
+  <si>
+    <t>% energy consumption (bev vs diesel)</t>
+  </si>
+  <si>
+    <t>from https://static1.squarespace.com/static/5eab584a296dca09a66e85a6/t/627946f6c12c786debe434c7/1652115191705/TCO_report_May%2B2022.pdf</t>
+  </si>
+  <si>
+    <t>e-tractor</t>
+  </si>
+  <si>
+    <t>IC</t>
+  </si>
+  <si>
+    <t>capital cost</t>
+  </si>
+  <si>
+    <t>operating hours/yr</t>
+  </si>
+  <si>
+    <t>Annual energy (gal)</t>
+  </si>
+  <si>
+    <t>Annual energy (kWh)</t>
+  </si>
+  <si>
+    <t>** costs in table 3</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>Annual usage (hr)</t>
+  </si>
+  <si>
+    <t>2022 to 2012 USD</t>
+  </si>
+  <si>
+    <t>PIFURfE for ag tractors (other processes)</t>
+  </si>
+  <si>
+    <t>Electric</t>
+  </si>
+  <si>
+    <t>price ($)</t>
+  </si>
+  <si>
+    <t>annual E</t>
+  </si>
+  <si>
+    <t>Assumed annual usage (hours)</t>
+  </si>
+  <si>
+    <t>E intensity (BTU/hr)</t>
+  </si>
+  <si>
+    <t>^assuming equal distribution of tasks</t>
+  </si>
+  <si>
+    <t>Annual BTUs</t>
+  </si>
+  <si>
+    <t>2021 to 2012 USD</t>
+  </si>
+  <si>
+    <t>Annual BTU</t>
+  </si>
+  <si>
+    <t>Diesel tractor price $/BTU</t>
+  </si>
+  <si>
+    <t>Electric tractor price $/BTU</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -1383,7 +1527,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1447,6 +1591,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1541,7 +1691,7 @@
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1626,6 +1776,12 @@
     <xf numFmtId="11" fontId="8" fillId="11" borderId="3" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="9" fontId="8" fillId="11" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2754,6 +2910,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2761,7 +2918,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3472,6 +3628,187 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>675943</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>88899</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2B59920-8ABB-1873-C7FA-CDD37215352D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="7429499"/>
+          <a:ext cx="4889168" cy="2752725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>139700</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>12504</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D28FB0B8-005B-4E65-A536-DC3EBE8AE389}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5934075" y="7429500"/>
+          <a:ext cx="4410075" cy="3254179"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>610454</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>76742</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2043415-C480-F862-EB46-E9D9439E8102}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="16002000"/>
+          <a:ext cx="6115904" cy="3886742"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>320866</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>38159</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{39C0BD5E-985B-0A39-B21D-7CCDBBB09B7B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="133350" y="13011150"/>
+          <a:ext cx="3721291" cy="1143059"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -3842,7 +4179,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC3CA314-6128-4FC9-9CED-BF85AF9DB226}">
-  <dimension ref="A1:B138"/>
+  <dimension ref="A1:B149"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="76.42578125" customWidth="1"/>
@@ -4351,24 +4688,66 @@
         <v>157</v>
       </c>
     </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B134" s="16" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B135" s="15" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B137" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B138" s="15" t="s">
         <v>186</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>138490</v>
+      </c>
+      <c r="B143" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>3412.14</v>
+      </c>
+      <c r="B145" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>0.78452102304761584</v>
+      </c>
+      <c r="B148" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>0.84730412960844359</v>
+      </c>
+      <c r="B149" t="s">
+        <v>446</v>
       </c>
     </row>
   </sheetData>
@@ -4392,6 +4771,651 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId17"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC78963D-3265-44FA-8138-35C2A57258D3}">
+  <sheetPr>
+    <tabColor theme="3" tint="0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1:M44"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="11" width="13.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="12">
+        <f>Boilers!$A$18</f>
+        <v>5.6711966224873446E-5</v>
+      </c>
+      <c r="C2" s="12">
+        <f>Boilers!$G$43</f>
+        <v>1.4986595988547842E-5</v>
+      </c>
+      <c r="D2" s="12">
+        <f>Boilers!A39</f>
+        <v>1.5989491110961776E-5</v>
+      </c>
+      <c r="E2" s="10">
+        <f>C2</f>
+        <v>1.4986595988547842E-5</v>
+      </c>
+      <c r="F2" s="12">
+        <f>Boilers!$G$44</f>
+        <v>9.436004881678272E-6</v>
+      </c>
+      <c r="G2" s="40">
+        <v>0</v>
+      </c>
+      <c r="H2" s="10">
+        <f>F2</f>
+        <v>9.436004881678272E-6</v>
+      </c>
+      <c r="I2" s="10">
+        <f>F2</f>
+        <v>9.436004881678272E-6</v>
+      </c>
+      <c r="J2" s="10">
+        <f>F2</f>
+        <v>9.436004881678272E-6</v>
+      </c>
+      <c r="K2" s="12">
+        <f>Boilers!A60</f>
+        <v>2.3984236666442662E-5</v>
+      </c>
+      <c r="L2" s="12">
+        <f>K2</f>
+        <v>2.3984236666442662E-5</v>
+      </c>
+      <c r="M2" s="12">
+        <f t="shared" ref="M2:M9" si="0">L2</f>
+        <v>2.3984236666442662E-5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="10">
+        <f>B2</f>
+        <v>5.6711966224873446E-5</v>
+      </c>
+      <c r="C3" s="10">
+        <f t="shared" ref="C3:K3" si="1">C2</f>
+        <v>1.4986595988547842E-5</v>
+      </c>
+      <c r="D3" s="10">
+        <f t="shared" si="1"/>
+        <v>1.5989491110961776E-5</v>
+      </c>
+      <c r="E3" s="10">
+        <f t="shared" si="1"/>
+        <v>1.4986595988547842E-5</v>
+      </c>
+      <c r="F3" s="10">
+        <f t="shared" si="1"/>
+        <v>9.436004881678272E-6</v>
+      </c>
+      <c r="G3" s="40">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H3" s="10">
+        <f t="shared" si="1"/>
+        <v>9.436004881678272E-6</v>
+      </c>
+      <c r="I3" s="10">
+        <f t="shared" si="1"/>
+        <v>9.436004881678272E-6</v>
+      </c>
+      <c r="J3" s="10">
+        <f t="shared" si="1"/>
+        <v>9.436004881678272E-6</v>
+      </c>
+      <c r="K3" s="10">
+        <f t="shared" si="1"/>
+        <v>2.3984236666442662E-5</v>
+      </c>
+      <c r="L3" s="10">
+        <f t="shared" ref="L3" si="2">K3</f>
+        <v>2.3984236666442662E-5</v>
+      </c>
+      <c r="M3" s="10">
+        <f t="shared" si="0"/>
+        <v>2.3984236666442662E-5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="12">
+        <f>'NB Medium Temp'!D40</f>
+        <v>3.4771933032458345E-5</v>
+      </c>
+      <c r="C4" s="10">
+        <f>D4</f>
+        <v>3.1780367029653324E-5</v>
+      </c>
+      <c r="D4" s="12">
+        <f>'NB Medium Temp'!D41</f>
+        <v>3.1780367029653324E-5</v>
+      </c>
+      <c r="E4" s="10">
+        <f>C4</f>
+        <v>3.1780367029653324E-5</v>
+      </c>
+      <c r="F4" s="10">
+        <f>D4</f>
+        <v>3.1780367029653324E-5</v>
+      </c>
+      <c r="G4" s="40">
+        <v>0</v>
+      </c>
+      <c r="H4" s="10">
+        <f t="shared" ref="H4" si="3">F4</f>
+        <v>3.1780367029653324E-5</v>
+      </c>
+      <c r="I4" s="10">
+        <f t="shared" ref="I4" si="4">F4</f>
+        <v>3.1780367029653324E-5</v>
+      </c>
+      <c r="J4" s="10">
+        <f t="shared" ref="J4" si="5">F4</f>
+        <v>3.1780367029653324E-5</v>
+      </c>
+      <c r="K4" s="10">
+        <f>D4</f>
+        <v>3.1780367029653324E-5</v>
+      </c>
+      <c r="L4" s="10">
+        <f t="shared" ref="L4" si="6">K4</f>
+        <v>3.1780367029653324E-5</v>
+      </c>
+      <c r="M4" s="10">
+        <f t="shared" si="0"/>
+        <v>3.1780367029653324E-5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="12">
+        <f>'NB High Temp'!F10</f>
+        <v>1.7204637228083889E-4</v>
+      </c>
+      <c r="C5" s="12">
+        <f>'NB High Temp'!F45</f>
+        <v>4.5951806950193628E-6</v>
+      </c>
+      <c r="D5" s="12">
+        <f>'NB High Temp'!F56</f>
+        <v>2.0725243194734525E-5</v>
+      </c>
+      <c r="E5" s="10">
+        <f>C5</f>
+        <v>4.5951806950193628E-6</v>
+      </c>
+      <c r="F5" s="10">
+        <f>D5*(F2/D2)</f>
+        <v>1.2230751723262388E-5</v>
+      </c>
+      <c r="G5" s="40">
+        <v>0</v>
+      </c>
+      <c r="H5" s="10">
+        <f t="shared" ref="H5" si="7">F5</f>
+        <v>1.2230751723262388E-5</v>
+      </c>
+      <c r="I5" s="10">
+        <f t="shared" ref="I5" si="8">F5</f>
+        <v>1.2230751723262388E-5</v>
+      </c>
+      <c r="J5" s="10">
+        <f t="shared" ref="J5" si="9">F5</f>
+        <v>1.2230751723262388E-5</v>
+      </c>
+      <c r="K5" s="12">
+        <f>'NB High Temp'!F67</f>
+        <v>3.265784625690839E-5</v>
+      </c>
+      <c r="L5" s="12">
+        <f t="shared" ref="L5" si="10">K5</f>
+        <v>3.265784625690839E-5</v>
+      </c>
+      <c r="M5" s="12">
+        <f t="shared" si="0"/>
+        <v>3.265784625690839E-5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="12">
+        <f>Cooling!$B$49</f>
+        <v>4.4520366169683022E-5</v>
+      </c>
+      <c r="C6" s="10">
+        <f>$D$6</f>
+        <v>1.8088159747275158E-5</v>
+      </c>
+      <c r="D6" s="12">
+        <f>Cooling!$B$27</f>
+        <v>1.8088159747275158E-5</v>
+      </c>
+      <c r="E6" s="10">
+        <f t="shared" ref="E6:F6" si="11">$D$6</f>
+        <v>1.8088159747275158E-5</v>
+      </c>
+      <c r="F6" s="10">
+        <f t="shared" si="11"/>
+        <v>1.8088159747275158E-5</v>
+      </c>
+      <c r="G6" s="40">
+        <v>0</v>
+      </c>
+      <c r="H6" s="10">
+        <f t="shared" ref="H6:J6" si="12">$D$6</f>
+        <v>1.8088159747275158E-5</v>
+      </c>
+      <c r="I6" s="10">
+        <f t="shared" si="12"/>
+        <v>1.8088159747275158E-5</v>
+      </c>
+      <c r="J6" s="10">
+        <f t="shared" si="12"/>
+        <v>1.8088159747275158E-5</v>
+      </c>
+      <c r="K6" s="10">
+        <f>$D$6*(K2/D2)</f>
+        <v>2.7132239620912736E-5</v>
+      </c>
+      <c r="L6" s="10">
+        <f t="shared" ref="L6" si="13">K6</f>
+        <v>2.7132239620912736E-5</v>
+      </c>
+      <c r="M6" s="10">
+        <f t="shared" si="0"/>
+        <v>2.7132239620912736E-5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="12">
+        <f>'Machine Drive'!$W$22</f>
+        <v>2.9652197760109964E-5</v>
+      </c>
+      <c r="C7" s="10">
+        <f>$F$7</f>
+        <v>7.0734511678239686E-5</v>
+      </c>
+      <c r="D7" s="10">
+        <f t="shared" ref="D7:E7" si="14">$F$7</f>
+        <v>7.0734511678239686E-5</v>
+      </c>
+      <c r="E7" s="10">
+        <f t="shared" si="14"/>
+        <v>7.0734511678239686E-5</v>
+      </c>
+      <c r="F7" s="12">
+        <f>'Machine Drive'!D38</f>
+        <v>7.0734511678239686E-5</v>
+      </c>
+      <c r="G7" s="40">
+        <v>0</v>
+      </c>
+      <c r="H7" s="10">
+        <f t="shared" ref="H7:K7" si="15">$F$7</f>
+        <v>7.0734511678239686E-5</v>
+      </c>
+      <c r="I7" s="10">
+        <f t="shared" si="15"/>
+        <v>7.0734511678239686E-5</v>
+      </c>
+      <c r="J7" s="10">
+        <f t="shared" si="15"/>
+        <v>7.0734511678239686E-5</v>
+      </c>
+      <c r="K7" s="10">
+        <f t="shared" si="15"/>
+        <v>7.0734511678239686E-5</v>
+      </c>
+      <c r="L7" s="10">
+        <f t="shared" ref="L7" si="16">K7</f>
+        <v>7.0734511678239686E-5</v>
+      </c>
+      <c r="M7" s="10">
+        <f t="shared" si="0"/>
+        <v>7.0734511678239686E-5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="12">
+        <f>Electrochemical!$G32</f>
+        <v>4.4539618429716232E-5</v>
+      </c>
+      <c r="C8" s="40">
+        <v>0</v>
+      </c>
+      <c r="D8" s="40">
+        <v>0</v>
+      </c>
+      <c r="E8" s="40">
+        <v>0</v>
+      </c>
+      <c r="F8" s="40">
+        <v>0</v>
+      </c>
+      <c r="G8" s="40">
+        <v>0</v>
+      </c>
+      <c r="H8" s="40">
+        <v>0</v>
+      </c>
+      <c r="I8" s="40">
+        <v>0</v>
+      </c>
+      <c r="J8" s="40">
+        <v>0</v>
+      </c>
+      <c r="K8" s="40">
+        <v>0</v>
+      </c>
+      <c r="L8" s="40">
+        <f t="shared" ref="L8" si="17">K8</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="40">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="12">
+        <f>Other!E9</f>
+        <v>7.0401933942914745E-6</v>
+      </c>
+      <c r="C9" s="10">
+        <f>D9*(C2/D2)</f>
+        <v>2.0886792055175448E-5</v>
+      </c>
+      <c r="D9" s="12">
+        <f>Other!B24</f>
+        <v>2.2284525195577483E-5</v>
+      </c>
+      <c r="E9" s="10">
+        <f>C9</f>
+        <v>2.0886792055175448E-5</v>
+      </c>
+      <c r="F9" s="10">
+        <f>D9*(F2/D2)</f>
+        <v>1.3150943145851209E-5</v>
+      </c>
+      <c r="G9" s="40">
+        <v>0</v>
+      </c>
+      <c r="H9" s="10">
+        <f>F9</f>
+        <v>1.3150943145851209E-5</v>
+      </c>
+      <c r="I9" s="10">
+        <f>F9</f>
+        <v>1.3150943145851209E-5</v>
+      </c>
+      <c r="J9" s="10">
+        <f>F9</f>
+        <v>1.3150943145851209E-5</v>
+      </c>
+      <c r="K9" s="10">
+        <f>D9*(K2/D2)</f>
+        <v>3.3426787793366228E-5</v>
+      </c>
+      <c r="L9" s="10">
+        <f t="shared" ref="L9" si="18">K9</f>
+        <v>3.3426787793366228E-5</v>
+      </c>
+      <c r="M9" s="10">
+        <f t="shared" si="0"/>
+        <v>3.3426787793366228E-5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B11" s="9"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>399</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="H3:J3 E3 D6" formula="1"/>
+  </ignoredErrors>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{843ADA01-EFFE-45B2-B6A7-C20F6BBCF0E2}">
+  <sheetPr>
+    <tabColor theme="3" tint="0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="13" width="13.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12">
+        <f>'Other (mobile)'!A7</f>
+        <v>3.1381977460259781E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10">
+        <f>B6</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="10">
+        <f>B6</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10">
+        <f>B6</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10">
+        <f>'Other (mobile)'!A6</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="10">
+        <f>B6</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="10">
+        <f>B6</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="10">
+        <f>B6</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="10">
+        <f>B6</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>401</v>
+      </c>
+      <c r="B12" s="10">
+        <f>B11</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>402</v>
+      </c>
+      <c r="B13" s="10">
+        <f>B12</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -6987,25 +8011,25 @@
       <c r="T23" s="21"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C24" s="55" t="s">
+      <c r="C24" s="61" t="s">
         <v>391</v>
       </c>
-      <c r="D24" s="56"/>
-      <c r="E24" s="57"/>
-      <c r="F24" s="52">
+      <c r="D24" s="62"/>
+      <c r="E24" s="63"/>
+      <c r="F24" s="58">
         <f>0.048/0.581</f>
         <v>8.2616179001721177E-2</v>
       </c>
-      <c r="G24" s="53"/>
-      <c r="H24" s="54"/>
-      <c r="I24" s="58">
+      <c r="G24" s="59"/>
+      <c r="H24" s="60"/>
+      <c r="I24" s="64">
         <f>((T13+T15)/2)</f>
         <v>23.414850000000001</v>
       </c>
-      <c r="J24" s="59"/>
-      <c r="K24" s="59"/>
-      <c r="L24" s="59"/>
-      <c r="M24" s="60"/>
+      <c r="J24" s="65"/>
+      <c r="K24" s="65"/>
+      <c r="L24" s="65"/>
+      <c r="M24" s="66"/>
       <c r="N24" s="51">
         <f>((W13+W15)/2)</f>
         <v>2.2407199119595664E-4</v>
@@ -7015,25 +8039,25 @@
       <c r="T24" s="21"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C25" s="55" t="s">
+      <c r="C25" s="61" t="s">
         <v>392</v>
       </c>
-      <c r="D25" s="56"/>
-      <c r="E25" s="57"/>
-      <c r="F25" s="52">
+      <c r="D25" s="62"/>
+      <c r="E25" s="63"/>
+      <c r="F25" s="58">
         <f>0.104/0.581</f>
         <v>0.17900172117039587</v>
       </c>
-      <c r="G25" s="53"/>
-      <c r="H25" s="54"/>
-      <c r="I25" s="58">
+      <c r="G25" s="59"/>
+      <c r="H25" s="60"/>
+      <c r="I25" s="64">
         <f>T14</f>
         <v>97.18877280000001</v>
       </c>
-      <c r="J25" s="59"/>
-      <c r="K25" s="59"/>
-      <c r="L25" s="59"/>
-      <c r="M25" s="60"/>
+      <c r="J25" s="65"/>
+      <c r="K25" s="65"/>
+      <c r="L25" s="65"/>
+      <c r="M25" s="66"/>
       <c r="N25" s="51">
         <f>W14</f>
         <v>3.3521233224690123E-5</v>
@@ -7043,25 +8067,25 @@
       <c r="T25" s="21"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C26" s="55" t="s">
+      <c r="C26" s="61" t="s">
         <v>390</v>
       </c>
-      <c r="D26" s="56"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="52">
+      <c r="D26" s="62"/>
+      <c r="E26" s="63"/>
+      <c r="F26" s="58">
         <f>0.127/0.581</f>
         <v>0.21858864027538727</v>
       </c>
-      <c r="G26" s="53"/>
-      <c r="H26" s="54"/>
-      <c r="I26" s="58">
+      <c r="G26" s="59"/>
+      <c r="H26" s="60"/>
+      <c r="I26" s="64">
         <f>T16</f>
         <v>319.17554000000001</v>
       </c>
-      <c r="J26" s="59"/>
-      <c r="K26" s="59"/>
-      <c r="L26" s="59"/>
-      <c r="M26" s="60"/>
+      <c r="J26" s="65"/>
+      <c r="K26" s="65"/>
+      <c r="L26" s="65"/>
+      <c r="M26" s="66"/>
       <c r="N26" s="51">
         <f>W16</f>
         <v>1.1301491868138288E-5</v>
@@ -7071,25 +8095,25 @@
       <c r="T26" s="21"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C27" s="55" t="s">
+      <c r="C27" s="61" t="s">
         <v>389</v>
       </c>
-      <c r="D27" s="56"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="52">
+      <c r="D27" s="62"/>
+      <c r="E27" s="63"/>
+      <c r="F27" s="58">
         <f>0.144/0.581</f>
         <v>0.24784853700516352</v>
       </c>
-      <c r="G27" s="53"/>
-      <c r="H27" s="54"/>
-      <c r="I27" s="58">
+      <c r="G27" s="59"/>
+      <c r="H27" s="60"/>
+      <c r="I27" s="64">
         <f>((T10+T18)/2)</f>
         <v>1214.1039020000001</v>
       </c>
-      <c r="J27" s="59"/>
-      <c r="K27" s="59"/>
-      <c r="L27" s="59"/>
-      <c r="M27" s="60"/>
+      <c r="J27" s="65"/>
+      <c r="K27" s="65"/>
+      <c r="L27" s="65"/>
+      <c r="M27" s="66"/>
       <c r="N27" s="51">
         <f>((W10+W18)/2)</f>
         <v>5.481183696812177E-6</v>
@@ -7099,25 +8123,25 @@
       <c r="T27" s="21"/>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C28" s="55" t="s">
+      <c r="C28" s="61" t="s">
         <v>393</v>
       </c>
-      <c r="D28" s="56"/>
-      <c r="E28" s="57"/>
-      <c r="F28" s="52">
+      <c r="D28" s="62"/>
+      <c r="E28" s="63"/>
+      <c r="F28" s="58">
         <f>0.157/0.581</f>
         <v>0.27022375215146299</v>
       </c>
-      <c r="G28" s="53"/>
-      <c r="H28" s="54"/>
-      <c r="I28" s="58">
+      <c r="G28" s="59"/>
+      <c r="H28" s="60"/>
+      <c r="I28" s="64">
         <f>((T9+T11+T12+T17+T19)/5)</f>
         <v>49678.416604960003</v>
       </c>
-      <c r="J28" s="59"/>
-      <c r="K28" s="59"/>
-      <c r="L28" s="59"/>
-      <c r="M28" s="60"/>
+      <c r="J28" s="65"/>
+      <c r="K28" s="65"/>
+      <c r="L28" s="65"/>
+      <c r="M28" s="66"/>
       <c r="N28" s="51">
         <f>((W9+W11+W12+W17+W19)/5)</f>
         <v>4.8514850079979492E-6</v>
@@ -7721,502 +8745,441 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC78963D-3265-44FA-8138-35C2A57258D3}">
-  <sheetPr>
-    <tabColor theme="3" tint="0.249977111117893"/>
-  </sheetPr>
-  <dimension ref="A1:M44"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B88B710-1DAB-47E6-AE70-A12C5CA0B896}">
+  <dimension ref="A2:P84"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="11" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="2" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="53" t="s">
+        <v>404</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
+      <c r="M2" s="52"/>
+      <c r="N2" s="52"/>
+      <c r="O2" s="52"/>
+      <c r="P2" s="52"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="54">
+        <v>0.57060049240377109</v>
+      </c>
+      <c r="B3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="54">
+        <f>4000/15</f>
+        <v>266.66666666666669</v>
+      </c>
+      <c r="B4" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="24"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="56">
+        <f>AVERAGE(O30,H40,H84)</f>
+        <v>8.2719018162705823E-4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="56">
+        <f>AVERAGE(O31,H41,H83)</f>
+        <v>3.1381977460259781E-3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="24"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="24" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>409</v>
+      </c>
+      <c r="D29" t="s">
+        <v>411</v>
+      </c>
+      <c r="E29" t="s">
+        <v>412</v>
+      </c>
+      <c r="F29" t="s">
+        <v>413</v>
+      </c>
+      <c r="G29" t="s">
+        <v>414</v>
+      </c>
+      <c r="H29" t="s">
+        <v>418</v>
+      </c>
+      <c r="I29" t="s">
+        <v>436</v>
+      </c>
+      <c r="M29" t="s">
+        <v>440</v>
+      </c>
+      <c r="N29" t="s">
+        <v>441</v>
+      </c>
+      <c r="O29" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>406</v>
+      </c>
+      <c r="C30">
+        <v>17000</v>
+      </c>
+      <c r="D30">
+        <v>7.1</v>
+      </c>
+      <c r="F30">
+        <v>9.5</v>
+      </c>
+      <c r="G30" s="21">
+        <f>D30*About!$A$143</f>
+        <v>983279</v>
+      </c>
+      <c r="H30" s="21">
+        <f>G30/F30</f>
+        <v>103503.05263157895</v>
+      </c>
+      <c r="I30">
+        <v>250</v>
+      </c>
+      <c r="L30" t="s">
+        <v>403</v>
+      </c>
+      <c r="M30">
+        <f>AVERAGE(C30:C32)*About!A148</f>
+        <v>21966.588645333242</v>
+      </c>
+      <c r="N30">
+        <f>AVERAGE(H30:H32)*A4</f>
+        <v>27574616.079328757</v>
+      </c>
+      <c r="O30" s="55">
+        <f>M30/N30</f>
+        <v>7.9662355342094654E-4</v>
+      </c>
+    </row>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>407</v>
+      </c>
+      <c r="C31">
+        <v>17000</v>
+      </c>
+      <c r="D31">
+        <v>7.1</v>
+      </c>
+      <c r="F31">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>401</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="12">
-        <f>Boilers!$A$18</f>
-        <v>5.6711966224873446E-5</v>
-      </c>
-      <c r="C2" s="12">
-        <f>Boilers!$G$43</f>
-        <v>1.4986595988547842E-5</v>
-      </c>
-      <c r="D2" s="12">
-        <f>Boilers!A39</f>
-        <v>1.5989491110961776E-5</v>
-      </c>
-      <c r="E2" s="10">
-        <f>C2</f>
-        <v>1.4986595988547842E-5</v>
-      </c>
-      <c r="F2" s="12">
-        <f>Boilers!$G$44</f>
-        <v>9.436004881678272E-6</v>
-      </c>
-      <c r="G2" s="40">
-        <v>0</v>
-      </c>
-      <c r="H2" s="10">
-        <f>F2</f>
-        <v>9.436004881678272E-6</v>
-      </c>
-      <c r="I2" s="10">
-        <f>F2</f>
-        <v>9.436004881678272E-6</v>
-      </c>
-      <c r="J2" s="10">
-        <f>F2</f>
-        <v>9.436004881678272E-6</v>
-      </c>
-      <c r="K2" s="12">
-        <f>Boilers!A60</f>
-        <v>2.3984236666442662E-5</v>
-      </c>
-      <c r="L2" s="12">
-        <f>K2</f>
-        <v>2.3984236666442662E-5</v>
-      </c>
-      <c r="M2" s="12">
-        <f t="shared" ref="M2:M9" si="0">L2</f>
-        <v>2.3984236666442662E-5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="10">
-        <f>B2</f>
-        <v>5.6711966224873446E-5</v>
-      </c>
-      <c r="C3" s="10">
-        <f t="shared" ref="C3:K3" si="1">C2</f>
-        <v>1.4986595988547842E-5</v>
-      </c>
-      <c r="D3" s="10">
-        <f t="shared" si="1"/>
-        <v>1.5989491110961776E-5</v>
-      </c>
-      <c r="E3" s="10">
-        <f t="shared" si="1"/>
-        <v>1.4986595988547842E-5</v>
-      </c>
-      <c r="F3" s="10">
-        <f t="shared" si="1"/>
-        <v>9.436004881678272E-6</v>
-      </c>
-      <c r="G3" s="40">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H3" s="10">
-        <f t="shared" si="1"/>
-        <v>9.436004881678272E-6</v>
-      </c>
-      <c r="I3" s="10">
-        <f t="shared" si="1"/>
-        <v>9.436004881678272E-6</v>
-      </c>
-      <c r="J3" s="10">
-        <f t="shared" si="1"/>
-        <v>9.436004881678272E-6</v>
-      </c>
-      <c r="K3" s="10">
-        <f t="shared" si="1"/>
-        <v>2.3984236666442662E-5</v>
-      </c>
-      <c r="L3" s="10">
-        <f t="shared" ref="L3:M3" si="2">K3</f>
-        <v>2.3984236666442662E-5</v>
-      </c>
-      <c r="M3" s="10">
+      <c r="G31" s="21">
+        <f>D31*About!$A$143</f>
+        <v>983279</v>
+      </c>
+      <c r="H31" s="21">
+        <f t="shared" ref="H31:H32" si="0">G31/F31</f>
+        <v>98327.9</v>
+      </c>
+      <c r="I31">
+        <v>250</v>
+      </c>
+      <c r="L31" t="s">
+        <v>439</v>
+      </c>
+      <c r="M31">
+        <f>C33*About!A148</f>
+        <v>43148.65626761887</v>
+      </c>
+      <c r="N31">
+        <f>N30*(1-A3)</f>
+        <v>11840526.566618824</v>
+      </c>
+      <c r="O31" s="55">
+        <f>M31/N31</f>
+        <v>3.6441501165383038E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>408</v>
+      </c>
+      <c r="C32">
+        <v>50000</v>
+      </c>
+      <c r="D32">
+        <v>18</v>
+      </c>
+      <c r="F32">
+        <v>23</v>
+      </c>
+      <c r="G32" s="21">
+        <f>D32*About!$A$143</f>
+        <v>2492820</v>
+      </c>
+      <c r="H32" s="21">
         <f t="shared" si="0"/>
-        <v>2.3984236666442662E-5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="12">
-        <f>'NB Medium Temp'!D40</f>
-        <v>3.4771933032458345E-5</v>
-      </c>
-      <c r="C4" s="10">
-        <f>D4</f>
-        <v>3.1780367029653324E-5</v>
-      </c>
-      <c r="D4" s="12">
-        <f>'NB Medium Temp'!D41</f>
-        <v>3.1780367029653324E-5</v>
-      </c>
-      <c r="E4" s="10">
-        <f>C4</f>
-        <v>3.1780367029653324E-5</v>
-      </c>
-      <c r="F4" s="10">
-        <f>D4</f>
-        <v>3.1780367029653324E-5</v>
-      </c>
-      <c r="G4" s="40">
-        <v>0</v>
-      </c>
-      <c r="H4" s="10">
-        <f t="shared" ref="H4" si="3">F4</f>
-        <v>3.1780367029653324E-5</v>
-      </c>
-      <c r="I4" s="10">
-        <f t="shared" ref="I4" si="4">F4</f>
-        <v>3.1780367029653324E-5</v>
-      </c>
-      <c r="J4" s="10">
-        <f t="shared" ref="J4" si="5">F4</f>
-        <v>3.1780367029653324E-5</v>
-      </c>
-      <c r="K4" s="10">
-        <f>D4</f>
-        <v>3.1780367029653324E-5</v>
-      </c>
-      <c r="L4" s="10">
-        <f t="shared" ref="L4:M4" si="6">K4</f>
-        <v>3.1780367029653324E-5</v>
-      </c>
-      <c r="M4" s="10">
-        <f t="shared" si="0"/>
-        <v>3.1780367029653324E-5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="12">
-        <f>'NB High Temp'!F10</f>
-        <v>1.7204637228083889E-4</v>
-      </c>
-      <c r="C5" s="12">
-        <f>'NB High Temp'!F45</f>
-        <v>4.5951806950193628E-6</v>
-      </c>
-      <c r="D5" s="12">
-        <f>'NB High Temp'!F56</f>
-        <v>2.0725243194734525E-5</v>
-      </c>
-      <c r="E5" s="10">
-        <f>C5</f>
-        <v>4.5951806950193628E-6</v>
-      </c>
-      <c r="F5" s="10">
-        <f>D5*(F2/D2)</f>
-        <v>1.2230751723262388E-5</v>
-      </c>
-      <c r="G5" s="40">
-        <v>0</v>
-      </c>
-      <c r="H5" s="10">
-        <f t="shared" ref="H5" si="7">F5</f>
-        <v>1.2230751723262388E-5</v>
-      </c>
-      <c r="I5" s="10">
-        <f t="shared" ref="I5" si="8">F5</f>
-        <v>1.2230751723262388E-5</v>
-      </c>
-      <c r="J5" s="10">
-        <f t="shared" ref="J5" si="9">F5</f>
-        <v>1.2230751723262388E-5</v>
-      </c>
-      <c r="K5" s="12">
-        <f>'NB High Temp'!F67</f>
-        <v>3.265784625690839E-5</v>
-      </c>
-      <c r="L5" s="12">
-        <f t="shared" ref="L5:M5" si="10">K5</f>
-        <v>3.265784625690839E-5</v>
-      </c>
-      <c r="M5" s="12">
-        <f t="shared" si="0"/>
-        <v>3.265784625690839E-5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="12">
-        <f>Cooling!$B$49</f>
-        <v>4.4520366169683022E-5</v>
-      </c>
-      <c r="C6" s="10">
-        <f>$D$6</f>
-        <v>1.8088159747275158E-5</v>
-      </c>
-      <c r="D6" s="12">
-        <f>Cooling!$B$27</f>
-        <v>1.8088159747275158E-5</v>
-      </c>
-      <c r="E6" s="10">
-        <f t="shared" ref="E6:F6" si="11">$D$6</f>
-        <v>1.8088159747275158E-5</v>
-      </c>
-      <c r="F6" s="10">
-        <f t="shared" si="11"/>
-        <v>1.8088159747275158E-5</v>
-      </c>
-      <c r="G6" s="40">
-        <v>0</v>
-      </c>
-      <c r="H6" s="10">
-        <f t="shared" ref="H6:J6" si="12">$D$6</f>
-        <v>1.8088159747275158E-5</v>
-      </c>
-      <c r="I6" s="10">
-        <f t="shared" si="12"/>
-        <v>1.8088159747275158E-5</v>
-      </c>
-      <c r="J6" s="10">
-        <f t="shared" si="12"/>
-        <v>1.8088159747275158E-5</v>
-      </c>
-      <c r="K6" s="10">
-        <f>$D$6*(K2/D2)</f>
-        <v>2.7132239620912736E-5</v>
-      </c>
-      <c r="L6" s="10">
-        <f t="shared" ref="L6:M6" si="13">K6</f>
-        <v>2.7132239620912736E-5</v>
-      </c>
-      <c r="M6" s="10">
-        <f t="shared" si="0"/>
-        <v>2.7132239620912736E-5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+        <v>108383.47826086957</v>
+      </c>
+      <c r="I32">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>410</v>
+      </c>
+      <c r="C33">
+        <v>55000</v>
+      </c>
+      <c r="E33">
+        <v>24</v>
+      </c>
+      <c r="F33">
         <v>16</v>
       </c>
-      <c r="B7" s="12">
-        <f>'Machine Drive'!$W$22</f>
-        <v>2.9652197760109964E-5</v>
-      </c>
-      <c r="C7" s="10">
-        <f>$F$7</f>
-        <v>7.0734511678239686E-5</v>
-      </c>
-      <c r="D7" s="10">
-        <f t="shared" ref="D7:E7" si="14">$F$7</f>
-        <v>7.0734511678239686E-5</v>
-      </c>
-      <c r="E7" s="10">
-        <f t="shared" si="14"/>
-        <v>7.0734511678239686E-5</v>
-      </c>
-      <c r="F7" s="12">
-        <f>'Machine Drive'!D38</f>
-        <v>7.0734511678239686E-5</v>
-      </c>
-      <c r="G7" s="40">
-        <v>0</v>
-      </c>
-      <c r="H7" s="10">
-        <f t="shared" ref="H7:M7" si="15">$F$7</f>
-        <v>7.0734511678239686E-5</v>
-      </c>
-      <c r="I7" s="10">
-        <f t="shared" si="15"/>
-        <v>7.0734511678239686E-5</v>
-      </c>
-      <c r="J7" s="10">
-        <f t="shared" si="15"/>
-        <v>7.0734511678239686E-5</v>
-      </c>
-      <c r="K7" s="10">
-        <f t="shared" si="15"/>
-        <v>7.0734511678239686E-5</v>
-      </c>
-      <c r="L7" s="10">
-        <f t="shared" ref="L7:M7" si="16">K7</f>
-        <v>7.0734511678239686E-5</v>
-      </c>
-      <c r="M7" s="10">
-        <f t="shared" si="0"/>
-        <v>7.0734511678239686E-5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="12">
-        <f>Electrochemical!$G32</f>
-        <v>4.4539618429716232E-5</v>
-      </c>
-      <c r="C8" s="40">
-        <v>0</v>
-      </c>
-      <c r="D8" s="40">
-        <v>0</v>
-      </c>
-      <c r="E8" s="40">
-        <v>0</v>
-      </c>
-      <c r="F8" s="40">
-        <v>0</v>
-      </c>
-      <c r="G8" s="40">
-        <v>0</v>
-      </c>
-      <c r="H8" s="40">
-        <v>0</v>
-      </c>
-      <c r="I8" s="40">
-        <v>0</v>
-      </c>
-      <c r="J8" s="40">
-        <v>0</v>
-      </c>
-      <c r="K8" s="40">
-        <v>0</v>
-      </c>
-      <c r="L8" s="40">
-        <f t="shared" ref="L8:M8" si="17">K8</f>
-        <v>0</v>
-      </c>
-      <c r="M8" s="40">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="12">
-        <f>Other!E9</f>
-        <v>7.0401933942914745E-6</v>
-      </c>
-      <c r="C9" s="10">
-        <f>D9*(C2/D2)</f>
-        <v>2.0886792055175448E-5</v>
-      </c>
-      <c r="D9" s="12">
-        <f>Other!B24</f>
-        <v>2.2284525195577483E-5</v>
-      </c>
-      <c r="E9" s="10">
-        <f>C9</f>
-        <v>2.0886792055175448E-5</v>
-      </c>
-      <c r="F9" s="10">
-        <f>D9*(F2/D2)</f>
-        <v>1.3150943145851209E-5</v>
-      </c>
-      <c r="G9" s="40">
-        <v>0</v>
-      </c>
-      <c r="H9" s="10">
-        <f>F9</f>
-        <v>1.3150943145851209E-5</v>
-      </c>
-      <c r="I9" s="10">
-        <f>F9</f>
-        <v>1.3150943145851209E-5</v>
-      </c>
-      <c r="J9" s="10">
-        <f>F9</f>
-        <v>1.3150943145851209E-5</v>
-      </c>
-      <c r="K9" s="10">
-        <f>D9*(K2/D2)</f>
-        <v>3.3426787793366228E-5</v>
-      </c>
-      <c r="L9" s="10">
-        <f t="shared" ref="L9:M9" si="18">K9</f>
-        <v>3.3426787793366228E-5</v>
-      </c>
-      <c r="M9" s="10">
-        <f t="shared" si="0"/>
-        <v>3.3426787793366228E-5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>399</v>
+      <c r="G33" s="21">
+        <f>E33*About!$A$145</f>
+        <v>81891.360000000001</v>
+      </c>
+      <c r="H33" s="21"/>
+      <c r="I33">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C34">
+        <f>C33/AVERAGE(C30:C32)</f>
+        <v>1.9642857142857142</v>
+      </c>
+      <c r="H34" s="21"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E35">
+        <f>E33/38.1</f>
+        <v>0.62992125984251968</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="24" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>420</v>
+      </c>
+      <c r="D39" t="s">
+        <v>247</v>
+      </c>
+      <c r="E39" t="s">
+        <v>435</v>
+      </c>
+      <c r="F39" t="s">
+        <v>443</v>
+      </c>
+      <c r="G39" t="s">
+        <v>445</v>
+      </c>
+      <c r="H39" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>421</v>
+      </c>
+      <c r="C40">
+        <v>2940</v>
+      </c>
+      <c r="D40">
+        <v>545</v>
+      </c>
+      <c r="E40">
+        <f>37500</f>
+        <v>37500</v>
+      </c>
+      <c r="F40" s="21">
+        <f>AVERAGE(60400,120900,214300)</f>
+        <v>131866.66666666666</v>
+      </c>
+      <c r="G40" s="21">
+        <f>F40*$A$4</f>
+        <v>35164444.444444448</v>
+      </c>
+      <c r="H40" s="55">
+        <f>E40*About!$A$149/G40</f>
+        <v>9.0358045924813471E-4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>422</v>
+      </c>
+      <c r="C41">
+        <v>113</v>
+      </c>
+      <c r="D41">
+        <v>995</v>
+      </c>
+      <c r="E41" s="21">
+        <f>AVERAGE(58000,74999)</f>
+        <v>66499.5</v>
+      </c>
+      <c r="F41" s="21">
+        <f>F40*(1-A3)</f>
+        <v>56623.481735022717</v>
+      </c>
+      <c r="G41" s="21">
+        <f>F41*$A$4</f>
+        <v>15099595.129339391</v>
+      </c>
+      <c r="H41" s="55">
+        <f>E41*About!$A$149/G41</f>
+        <v>3.7315769386037706E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F42" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="24" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C55" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>424</v>
+      </c>
+      <c r="C56" s="19">
+        <v>0.54</v>
+      </c>
+      <c r="E56" s="11" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>425</v>
+      </c>
+      <c r="C57" s="19">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C58" s="19"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="24" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="82" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C82" t="s">
+        <v>430</v>
+      </c>
+      <c r="D82" t="s">
+        <v>431</v>
+      </c>
+      <c r="E82" t="s">
+        <v>432</v>
+      </c>
+      <c r="F82" t="s">
+        <v>433</v>
+      </c>
+      <c r="G82" t="s">
+        <v>447</v>
+      </c>
+      <c r="H82" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="83" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B83" t="s">
+        <v>428</v>
+      </c>
+      <c r="C83">
+        <v>28398</v>
+      </c>
+      <c r="D83">
+        <v>250</v>
+      </c>
+      <c r="G83" s="21">
+        <f>G84*(1-A3)</f>
+        <v>11801531.10292552</v>
+      </c>
+      <c r="H83" s="55">
+        <f>C83*About!$A$149/G83</f>
+        <v>2.0388661829358595E-3</v>
+      </c>
+    </row>
+    <row r="84" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>429</v>
+      </c>
+      <c r="C84">
+        <v>25345</v>
+      </c>
+      <c r="D84">
+        <v>250</v>
+      </c>
+      <c r="E84">
+        <f>AVERAGE(144,228.1)</f>
+        <v>186.05</v>
+      </c>
+      <c r="G84" s="21">
+        <f>E84*About!A143*A4/D84</f>
+        <v>27483802.133333337</v>
+      </c>
+      <c r="H84" s="55">
+        <f>C84*About!$A$149/G84</f>
+        <v>7.8136653221209343E-4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="H3:J3 E3 D6" formula="1"/>
-  </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correcting some inaccurate labels in indst/IECCpUAEU (does not affect numerical results)
</commit_message>
<xml_diff>
--- a/InputData/indst/IECCpUAEU/Indst Eqpt Cap Cost per Unit Ann E Use.xlsx
+++ b/InputData/indst/IECCpUAEU/Indst Eqpt Cap Cost per Unit Ann E Use.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code Repositories\eps-us\InputData\indst\IECCpUAEU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B7C46AE-AD16-41EE-AF51-56BA6F443605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{048DA2A3-2C9E-4B97-876D-4CA04A490527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27690" yWindow="750" windowWidth="23940" windowHeight="21210" tabRatio="762" xr2:uid="{6A73F6BA-E2AF-4EFC-B7D0-AD586970A910}"/>
+    <workbookView xWindow="14145" yWindow="1035" windowWidth="33990" windowHeight="22305" tabRatio="762" xr2:uid="{6A73F6BA-E2AF-4EFC-B7D0-AD586970A910}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -123,9 +123,6 @@
     <t>other processes</t>
   </si>
   <si>
-    <t>Annual heat delivered (MMbtu)</t>
-  </si>
-  <si>
     <t>Capital Cost (USD)</t>
   </si>
   <si>
@@ -147,9 +144,6 @@
     <t>BTU</t>
   </si>
   <si>
-    <t>Capital cost per BTU</t>
-  </si>
-  <si>
     <t>$/(BTU/yr)</t>
   </si>
   <si>
@@ -246,9 +240,6 @@
     <t>50% more than a natural gas boiler.</t>
   </si>
   <si>
-    <t>Cost per annual energy ($/(BTU/yr))</t>
-  </si>
-  <si>
     <t>For electricity in the "boilers" end use, we use industrial heat pumps rather than electric boilers because industrial heat pumps</t>
   </si>
   <si>
@@ -534,12 +525,6 @@
     <t>Average total operating capacity (first 3 years)</t>
   </si>
   <si>
-    <t xml:space="preserve">Yield in kWh/year: </t>
-  </si>
-  <si>
-    <t>Yield in BTU/year</t>
-  </si>
-  <si>
     <t>DOE projected capex cost reduction by 2030:</t>
   </si>
   <si>
@@ -606,12 +591,6 @@
     <t>kWh/year</t>
   </si>
   <si>
-    <t>Annual heat delivered/year (mmBTU):</t>
-  </si>
-  <si>
-    <t>Annual energy expenditure/year (kWh):</t>
-  </si>
-  <si>
     <t>mmBTU/year</t>
   </si>
   <si>
@@ -844,9 +823,6 @@
   </si>
   <si>
     <t>Electric example (Infrared Heater for Processed Foods)</t>
-  </si>
-  <si>
-    <t>Energy expenditure:</t>
   </si>
   <si>
     <t>USD</t>
@@ -1192,9 +1168,6 @@
     </r>
   </si>
   <si>
-    <t>Annual energy delivered (MMbtu)</t>
-  </si>
-  <si>
     <t xml:space="preserve">% Distr. by Energy Use of Motor HP Category </t>
   </si>
   <si>
@@ -1231,9 +1204,6 @@
     <t>% Distr. by Energy Use Per HP Bin</t>
   </si>
   <si>
-    <t>Average Annual Energy Delivered by HP Bin (MMbtu)</t>
-  </si>
-  <si>
     <t>electrified industrial heating equipment. So we do not consider them to be an outlier - i.e., the higher cost is justified.</t>
   </si>
   <si>
@@ -1439,6 +1409,36 @@
   </si>
   <si>
     <t>Does not need to be converted using heat pump COP because it is already based on electricity consumption</t>
+  </si>
+  <si>
+    <t>Cost per annual energy input ($/(BTU/yr))</t>
+  </si>
+  <si>
+    <t>Capital cost per BTU energy consumption</t>
+  </si>
+  <si>
+    <t>Annual energy consumption/year (kWh):</t>
+  </si>
+  <si>
+    <t>Annual energy consumption/year (mmBTU):</t>
+  </si>
+  <si>
+    <t>Annual energy consumed (MMbtu)</t>
+  </si>
+  <si>
+    <t>Annual energy use (MMbtu)</t>
+  </si>
+  <si>
+    <t>Average Annual Energy Use by HP Bin (MMbtu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy use in kWh/year: </t>
+  </si>
+  <si>
+    <t>Energy use in BTU/year</t>
+  </si>
+  <si>
+    <t>Capacity:</t>
   </si>
 </sst>
 </file>
@@ -1695,7 +1695,7 @@
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1786,33 +1786,6 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="8" fillId="11" borderId="4" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="11" borderId="5" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="11" borderId="6" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="11" borderId="4" xfId="3" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="8" fillId="11" borderId="5" xfId="3" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="8" fillId="11" borderId="6" xfId="3" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="8" fillId="11" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="11" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="11" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1825,7 +1798,28 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="11" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="11" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="11" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="11" borderId="4" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="11" borderId="5" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="11" borderId="6" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="8" fillId="11" borderId="4" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="11" borderId="5" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="11" borderId="6" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3758,7 +3752,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>675943</xdr:colOff>
+      <xdr:colOff>523543</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>88899</xdr:rowOff>
     </xdr:to>
@@ -3846,7 +3840,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>610454</xdr:colOff>
+      <xdr:colOff>458054</xdr:colOff>
       <xdr:row>79</xdr:row>
       <xdr:rowOff>76742</xdr:rowOff>
     </xdr:to>
@@ -3890,7 +3884,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>320866</xdr:colOff>
+      <xdr:colOff>168466</xdr:colOff>
       <xdr:row>48</xdr:row>
       <xdr:rowOff>38159</xdr:rowOff>
     </xdr:to>
@@ -4308,7 +4302,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -4316,52 +4310,51 @@
         <v>0</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" s="68" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="67"/>
-      <c r="B4" s="69" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" s="68" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="67"/>
-      <c r="B5" s="70">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="13">
         <v>2025</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="68" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="67"/>
-      <c r="B6" s="69" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" s="68" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="67"/>
-      <c r="B7" s="71" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" s="68" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="67"/>
-      <c r="B8" s="69" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" s="68" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="67"/>
-      <c r="B9" s="69"/>
-    </row>
-    <row r="10" spans="1:2" s="68" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="67"/>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="58" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
       <c r="B10" s="16" t="s">
-        <v>433</v>
+        <v>423</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -4371,27 +4364,27 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" s="15" t="s">
-        <v>439</v>
+        <v>429</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>438</v>
+        <v>428</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="16" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
@@ -4401,27 +4394,27 @@
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="15" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="16" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.25">
@@ -4431,27 +4424,27 @@
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
@@ -4461,67 +4454,67 @@
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="15" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="16" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" s="16" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.25">
@@ -4531,22 +4524,22 @@
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
     </row>
     <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="15" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" s="16" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
     </row>
     <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
     </row>
     <row r="56" spans="2:2" x14ac:dyDescent="0.25">
@@ -4556,32 +4549,32 @@
     </row>
     <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" s="15" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
     </row>
     <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" s="16" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
     </row>
     <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" s="1" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
     </row>
     <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="64" spans="2:2" x14ac:dyDescent="0.25">
@@ -4591,12 +4584,12 @@
     </row>
     <row r="65" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B65" s="3" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="35" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.25">
@@ -4604,12 +4597,12 @@
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.25">
@@ -4619,17 +4612,17 @@
     </row>
     <row r="71" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B71" s="3" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
     </row>
     <row r="72" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B72" s="3" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="73" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B73" s="35" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="74" spans="2:2" x14ac:dyDescent="0.25">
@@ -4637,12 +4630,12 @@
     </row>
     <row r="75" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B75" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="76" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B76" s="3" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="77" spans="2:2" x14ac:dyDescent="0.25">
@@ -4652,12 +4645,12 @@
     </row>
     <row r="78" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B78" s="36" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="79" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B79" s="37" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.25">
@@ -4665,12 +4658,12 @@
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="1" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
     </row>
     <row r="83" spans="2:2" x14ac:dyDescent="0.25">
@@ -4680,7 +4673,7 @@
     </row>
     <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="15" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
     </row>
     <row r="85" spans="2:2" x14ac:dyDescent="0.25">
@@ -4688,7 +4681,7 @@
     </row>
     <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
     </row>
     <row r="87" spans="2:2" x14ac:dyDescent="0.25">
@@ -4698,22 +4691,22 @@
     </row>
     <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
     </row>
     <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="1" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
     </row>
     <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
     </row>
     <row r="93" spans="2:2" x14ac:dyDescent="0.25">
@@ -4723,27 +4716,27 @@
     </row>
     <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
     </row>
     <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="15" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
     </row>
     <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="31" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="36" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.25">
@@ -4753,12 +4746,12 @@
     </row>
     <row r="102" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B102" s="36" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="103" spans="2:2" ht="45" x14ac:dyDescent="0.25">
       <c r="B103" s="37" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="104" spans="2:2" x14ac:dyDescent="0.25">
@@ -4766,32 +4759,32 @@
     </row>
     <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="16" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="15" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="15" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="112" spans="2:2" x14ac:dyDescent="0.25">
@@ -4801,52 +4794,52 @@
     </row>
     <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="15" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
     </row>
     <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="15" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B135" s="16" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B136" s="15" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B138" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B139" s="15" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>398</v>
+        <v>388</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
@@ -4854,12 +4847,12 @@
         <v>138490</v>
       </c>
       <c r="B144" t="s">
-        <v>399</v>
+        <v>389</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>400</v>
+        <v>390</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
@@ -4867,7 +4860,7 @@
         <v>3412.14</v>
       </c>
       <c r="B146" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
@@ -4875,7 +4868,7 @@
         <v>0.78452102304761584</v>
       </c>
       <c r="B149" t="s">
-        <v>420</v>
+        <v>410</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
@@ -4883,7 +4876,7 @@
         <v>0.84730412960844359</v>
       </c>
       <c r="B150" t="s">
-        <v>429</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>
@@ -4925,7 +4918,7 @@
   <sheetData>
     <row r="1" spans="1:13" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -4958,10 +4951,10 @@
         <v>10</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -5378,32 +5371,32 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
     </row>
   </sheetData>
@@ -5429,7 +5422,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5535,7 +5528,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="B12" s="10">
         <f>B11</f>
@@ -5544,7 +5537,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="B13" s="10">
         <f>B12</f>
@@ -5567,13 +5560,13 @@
     <col min="4" max="4" width="18.42578125" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" customWidth="1"/>
-    <col min="7" max="7" width="20.28515625" customWidth="1"/>
+    <col min="7" max="7" width="22.28515625" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -5581,80 +5574,80 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="24" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="72" t="s">
-        <v>440</v>
-      </c>
-      <c r="B5" s="73" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="74" t="s">
+      <c r="A5" s="59" t="s">
+        <v>430</v>
+      </c>
+      <c r="B5" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="77"/>
+      <c r="C5" s="61" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="64"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>441</v>
+        <v>431</v>
       </c>
       <c r="B6">
         <v>600</v>
       </c>
-      <c r="C6" s="75" t="s">
-        <v>147</v>
+      <c r="C6" s="62" t="s">
+        <v>144</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>447</v>
+        <v>437</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>442</v>
+        <v>432</v>
       </c>
       <c r="B7">
         <v>8760</v>
       </c>
-      <c r="C7" s="75" t="s">
-        <v>443</v>
-      </c>
-      <c r="D7" s="75"/>
+      <c r="C7" s="62" t="s">
+        <v>433</v>
+      </c>
+      <c r="D7" s="62"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>444</v>
+        <v>434</v>
       </c>
       <c r="B8" s="19">
         <v>0.65</v>
       </c>
-      <c r="C8" s="75" t="s">
-        <v>154</v>
-      </c>
-      <c r="D8" s="75"/>
+      <c r="C8" s="62" t="s">
+        <v>151</v>
+      </c>
+      <c r="D8" s="62"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>445</v>
-      </c>
-      <c r="B9" s="76">
+        <v>435</v>
+      </c>
+      <c r="B9" s="63">
         <f>B6/(B7*B8)</f>
         <v>0.10537407797681771</v>
       </c>
-      <c r="C9" s="75" t="s">
-        <v>296</v>
+      <c r="C9" s="62" t="s">
+        <v>288</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>448</v>
+        <v>438</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -5662,13 +5655,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B11">
         <v>3412.14</v>
       </c>
-      <c r="C11" s="75" t="s">
-        <v>41</v>
+      <c r="C11" s="62" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -5676,28 +5669,28 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
       <c r="B13" s="12">
         <f>B9/B11</f>
         <v>3.0882108581950831E-5</v>
       </c>
-      <c r="C13" s="75" t="s">
-        <v>28</v>
+      <c r="C13" s="62" t="s">
+        <v>26</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>449</v>
+        <v>439</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="D14" s="24" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16" s="18"/>
       <c r="C16" s="18"/>
@@ -5706,12 +5699,12 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="B20" s="8">
         <v>80375</v>
@@ -5719,7 +5712,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="B21" s="8">
         <v>91475</v>
@@ -5727,7 +5720,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="B22" s="8">
         <f>AVERAGE(B20:B21)</f>
@@ -5736,7 +5729,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="B24">
         <v>400</v>
@@ -5744,7 +5737,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="B25">
         <v>0.74570000000000003</v>
@@ -5752,7 +5745,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B26">
         <f>B24*B25</f>
@@ -5761,7 +5754,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B28" s="22">
         <v>5280</v>
@@ -5769,42 +5762,42 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="B30">
         <f>B26*B28</f>
         <v>1574918.4000000001</v>
       </c>
       <c r="C30" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B31">
         <v>3412.14</v>
       </c>
       <c r="C31" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="B32">
         <f>B30*B31</f>
         <v>5373842069.3760004</v>
       </c>
       <c r="C32" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>27</v>
+        <v>442</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -5813,12 +5806,12 @@
         <v>1.5989491110961776E-5</v>
       </c>
       <c r="B35" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="17" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B37" s="18"/>
       <c r="C37" s="18"/>
@@ -5827,27 +5820,27 @@
     </row>
     <row r="38" spans="1:7" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="B38" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>60</v>
+        <v>441</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B39">
         <v>2000</v>
@@ -5873,7 +5866,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B40">
         <v>2000</v>
@@ -5899,7 +5892,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B41">
         <v>2000</v>
@@ -5925,60 +5918,60 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B43" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B44">
         <f>B39*B28</f>
         <v>10560000</v>
       </c>
       <c r="C44" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B45">
         <v>3412.14</v>
       </c>
       <c r="C45" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B46">
         <f>B44*B45</f>
         <v>36032198400</v>
       </c>
       <c r="C46" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="17" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B51" s="18"/>
       <c r="C51" s="18"/>
@@ -5986,13 +5979,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B53" s="8"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B54" s="20"/>
     </row>
@@ -6002,7 +5995,7 @@
         <v>2.3984236666442662E-5</v>
       </c>
       <c r="B56" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -6021,330 +6014,330 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B5" s="8">
         <v>307500</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B6">
         <v>4000</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B8" s="8">
         <v>75863</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B9" s="8">
         <v>6226</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B11" s="25">
         <v>0.45</v>
       </c>
       <c r="C11" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B12" s="25">
         <v>0.15</v>
       </c>
       <c r="C12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B14" s="21">
         <f>B8/B11</f>
         <v>168584.44444444444</v>
       </c>
       <c r="C14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B15" s="21">
         <f>B9/B12</f>
         <v>41506.666666666672</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B17">
         <v>100000</v>
       </c>
       <c r="C17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B18">
         <v>3412.14</v>
       </c>
       <c r="C18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B20" s="9">
         <f>B14*B17</f>
         <v>16858444444.444445</v>
       </c>
       <c r="C20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B21" s="9">
         <f>B15*B18</f>
         <v>141626557.60000002</v>
       </c>
       <c r="C21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B26" s="9">
         <f>SUM(B20:B21)</f>
         <v>17000071002.044445</v>
       </c>
       <c r="C26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B27" s="12">
         <f>B5/B26</f>
         <v>1.8088159747275158E-5</v>
       </c>
       <c r="C27" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B32" s="8">
         <v>200</v>
       </c>
       <c r="C32" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B33" s="8">
         <v>500</v>
       </c>
       <c r="C33" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B34" s="8">
         <f>AVERAGE(B32:B33)</f>
         <v>350</v>
       </c>
       <c r="C34" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B36">
         <v>500</v>
       </c>
       <c r="C36" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D36" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B38" s="8">
         <f>B34*B36</f>
         <v>175000</v>
       </c>
       <c r="C38" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B41">
         <v>0.57599999999999996</v>
       </c>
       <c r="C41" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B42">
         <f>B41*B36</f>
         <v>288</v>
       </c>
       <c r="C42" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B44">
         <f>B6</f>
         <v>4000</v>
       </c>
       <c r="C44" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D44" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B46">
         <f>B42*B44</f>
         <v>1152000</v>
       </c>
       <c r="C46" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B47" s="9">
         <f>B46*B18</f>
         <v>3930785280</v>
       </c>
       <c r="C47" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B49" s="12">
         <f>B38/B47</f>
         <v>4.4520366169683022E-5</v>
       </c>
       <c r="C49" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -6368,7 +6361,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -6376,25 +6369,25 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="41" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="B3" s="42"/>
       <c r="C3" s="11" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>319</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>327</v>
       </c>
       <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="B5">
         <v>492000</v>
@@ -6403,7 +6396,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="B6">
         <v>135000</v>
@@ -6412,7 +6405,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="B7">
         <v>474000</v>
@@ -6421,7 +6414,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="B8">
         <v>70000</v>
@@ -6430,7 +6423,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="B9">
         <v>22000</v>
@@ -6439,7 +6432,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="B10">
         <v>18000</v>
@@ -6448,7 +6441,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="B11">
         <v>216000</v>
@@ -6457,7 +6450,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="B12">
         <v>51000</v>
@@ -6466,7 +6459,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="B13">
         <v>125000</v>
@@ -6475,24 +6468,24 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="B15" s="42"/>
       <c r="C15" s="11" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="B17" s="20">
         <v>13400</v>
@@ -6500,7 +6493,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="B18" s="20">
         <v>5300</v>
@@ -6508,7 +6501,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="B19" s="20">
         <v>13600</v>
@@ -6516,32 +6509,32 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="41" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="B21" s="42"/>
       <c r="C21" s="42"/>
       <c r="D21" s="42"/>
       <c r="E21" s="11" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="B23">
         <v>4380</v>
@@ -6552,7 +6545,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="B24">
         <v>4380</v>
@@ -6563,7 +6556,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="B27" s="40"/>
       <c r="C27" s="40"/>
@@ -6571,32 +6564,32 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="B33" s="1">
         <f>'Boilers &amp; Heat Pumps'!B28</f>
@@ -6605,13 +6598,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B36" s="46">
         <v>3412.14</v>
       </c>
       <c r="C36" s="40" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -6619,7 +6612,7 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="45" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="B38" s="44"/>
       <c r="C38" s="44"/>
@@ -6627,21 +6620,21 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="B40">
         <f>$B$33*D23*B36</f>
@@ -6658,7 +6651,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="B41">
         <f>$B$33*C24</f>
@@ -6675,33 +6668,33 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="41" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="B51" s="42"/>
       <c r="C51" s="42"/>
       <c r="D51" s="11" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="B53">
         <v>722000</v>
@@ -6713,7 +6706,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="B54">
         <v>882000</v>
@@ -6741,7 +6734,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -6752,12 +6745,12 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I2" s="1" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C3" s="25"/>
       <c r="F3" s="25">
@@ -6765,107 +6758,107 @@
         <v>264.16000000000003</v>
       </c>
       <c r="G3" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="F4">
         <v>450</v>
       </c>
       <c r="G4" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C5" s="32"/>
       <c r="F5" s="32">
         <v>800000</v>
       </c>
       <c r="G5" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>181</v>
+        <v>443</v>
       </c>
       <c r="F7">
         <f>F4*F5</f>
         <v>360000000</v>
       </c>
       <c r="G7" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>180</v>
+        <v>444</v>
       </c>
       <c r="F8">
         <f>F7*0.003412</f>
         <v>1228320</v>
       </c>
       <c r="G8" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="F9" s="25">
         <f>F3*F5</f>
         <v>211328000.00000003</v>
       </c>
       <c r="G9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="F10" s="12">
         <f>F9/(F8*10^6)</f>
         <v>1.7204637228083889E-4</v>
       </c>
       <c r="G10" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="E12">
         <f>8760*155</f>
         <v>1357800</v>
       </c>
       <c r="F12" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="18"/>
@@ -6876,13 +6869,13 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="F16" s="20">
         <v>170</v>
       </c>
       <c r="G16" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -6891,7 +6884,7 @@
         <v>26.356589147286826</v>
       </c>
       <c r="G17" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -6900,7 +6893,7 @@
         <v>9.4883645023316546E-2</v>
       </c>
       <c r="G18" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -6909,80 +6902,80 @@
         <v>2.7808805692648461E-5</v>
       </c>
       <c r="G19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="F21">
         <v>36000000</v>
       </c>
       <c r="G21" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="F22" s="20">
         <f>F21*0.14</f>
         <v>5040000.0000000009</v>
       </c>
       <c r="G22" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I22" s="15"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="F23">
         <f>AVERAGE(5.1,7.8)</f>
         <v>6.4499999999999993</v>
       </c>
       <c r="G23" t="s">
+        <v>218</v>
+      </c>
+      <c r="I23" t="s">
         <v>225</v>
-      </c>
-      <c r="I23" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="F24">
         <v>8000</v>
       </c>
       <c r="G24" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="F25">
         <v>600</v>
       </c>
       <c r="G25" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -6991,7 +6984,7 @@
         <v>3869.9999999999995</v>
       </c>
       <c r="G26" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="I26" s="15"/>
     </row>
@@ -7001,95 +6994,95 @@
         <v>1289999.9999999998</v>
       </c>
       <c r="G27" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="I27" s="15"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>181</v>
+        <v>443</v>
       </c>
       <c r="F28">
         <f>F27*277.778</f>
         <v>358333619.99999994</v>
       </c>
       <c r="G28" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="I28" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>180</v>
+        <v>444</v>
       </c>
       <c r="F29">
         <f>F28*0.003412</f>
         <v>1222634.3114399998</v>
       </c>
       <c r="G29" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="F30" s="12">
         <f>(F21*0.14)/(F29*10^6)</f>
         <v>4.1222464909102436E-6</v>
       </c>
       <c r="G30" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="I30" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="F34">
         <v>21.08</v>
       </c>
       <c r="G34" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="I34" s="15" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="F35">
         <v>0.76</v>
       </c>
       <c r="G35" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I35" s="15" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="F36" s="34">
         <f>F34*F35</f>
         <v>16.020799999999998</v>
       </c>
       <c r="G36" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -7097,7 +7090,7 @@
         <v>1.3284</v>
       </c>
       <c r="G37" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -7106,7 +7099,7 @@
         <v>21.282030719999998</v>
       </c>
       <c r="G38" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -7114,7 +7107,7 @@
         <v>1.32</v>
       </c>
       <c r="G39" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -7123,7 +7116,7 @@
         <v>28.092280550399998</v>
       </c>
       <c r="G40" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -7132,7 +7125,7 @@
         <v>4.3553923333953488</v>
       </c>
       <c r="G41" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -7140,7 +7133,7 @@
         <v>277.77800000000002</v>
       </c>
       <c r="G42" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -7149,7 +7142,7 @@
         <v>1.5679399856703368E-2</v>
       </c>
       <c r="G43" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -7157,7 +7150,7 @@
         <v>3412.14</v>
       </c>
       <c r="G44" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -7166,12 +7159,12 @@
         <v>4.5951806950193628E-6</v>
       </c>
       <c r="G45" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="B47" s="18"/>
       <c r="C47" s="18"/>
@@ -7182,99 +7175,99 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="F49" s="32">
         <v>6000000</v>
       </c>
       <c r="G49" s="33" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="I49" s="15" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="F50">
         <v>300</v>
       </c>
       <c r="G50" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="I50" s="15" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="F51">
         <v>8760</v>
       </c>
       <c r="G51" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="I51" s="15" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="F52">
         <v>1100</v>
       </c>
       <c r="G52" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="I52" s="15" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>181</v>
+        <v>443</v>
       </c>
       <c r="F54">
         <f>(F3*365)*F52</f>
         <v>106060240.00000001</v>
       </c>
       <c r="G54" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>180</v>
+        <v>444</v>
       </c>
       <c r="F55" s="34">
         <f>F54*0.003412</f>
         <v>361877.53888000007</v>
       </c>
       <c r="G55" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="F56" s="12">
         <f>(F49*1.25)/(F55*10^6)</f>
         <v>2.0725243194734525E-5</v>
       </c>
       <c r="G56" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="17" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="B58" s="18"/>
       <c r="C58" s="18"/>
@@ -7285,90 +7278,90 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="F60">
         <f>574-184</f>
         <v>390</v>
       </c>
       <c r="G60" s="33" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="F61">
         <v>3500</v>
       </c>
       <c r="G61" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="I61" s="15" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F62" s="32">
         <v>1500000</v>
       </c>
       <c r="G62" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="I62" s="15" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>181</v>
+        <v>443</v>
       </c>
       <c r="F64">
         <f>F61*F62</f>
         <v>5250000000</v>
       </c>
       <c r="G64" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>180</v>
+        <v>444</v>
       </c>
       <c r="F65">
         <f>F64*0.003412</f>
         <v>17913000</v>
       </c>
       <c r="G65" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="F66" s="25">
         <f>F60*F62</f>
         <v>585000000</v>
       </c>
       <c r="G66" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="F67" s="12">
         <f>F66/(F65*10^6)</f>
         <v>3.265784625690839E-5</v>
       </c>
       <c r="G67" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -7408,96 +7401,96 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="E8" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="F8" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="G8" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="H8" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="I8" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="G8" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="H8" s="26" t="s">
-        <v>124</v>
-      </c>
-      <c r="I8" s="26" t="s">
-        <v>125</v>
-      </c>
       <c r="J8" s="30" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="K8" s="27"/>
       <c r="L8" s="29" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="M8" s="27"/>
       <c r="N8" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O8" s="27"/>
       <c r="P8" s="29" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="Q8" s="27"/>
       <c r="R8" s="29" t="s">
-        <v>369</v>
+        <v>360</v>
       </c>
       <c r="S8" s="27"/>
       <c r="T8" s="29" t="s">
-        <v>368</v>
+        <v>446</v>
       </c>
       <c r="U8" s="27"/>
       <c r="V8" s="27"/>
       <c r="W8" s="29" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D9">
         <v>0.3</v>
@@ -7547,10 +7540,10 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D10">
         <v>8</v>
@@ -7600,10 +7593,10 @@
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D11">
         <v>350</v>
@@ -7653,10 +7646,10 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D12">
         <v>500</v>
@@ -7706,10 +7699,10 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C13" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D13">
         <v>0.35</v>
@@ -7759,10 +7752,10 @@
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D14">
         <v>1.8</v>
@@ -7812,10 +7805,10 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D15">
         <v>0.35</v>
@@ -7865,10 +7858,10 @@
     </row>
     <row r="16" spans="1:23" ht="30" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D16">
         <v>3</v>
@@ -7918,10 +7911,10 @@
     </row>
     <row r="17" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C17" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D17">
         <v>50</v>
@@ -7971,10 +7964,10 @@
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C18" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D18">
         <v>3</v>
@@ -8024,10 +8017,10 @@
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D19">
         <v>180</v>
@@ -8080,7 +8073,7 @@
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="N21" s="21"/>
       <c r="P21" s="21"/>
@@ -8096,7 +8089,7 @@
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="N22" s="21"/>
       <c r="P22" s="21"/>
@@ -8114,49 +8107,49 @@
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C23" s="49" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
       <c r="D23" s="49"/>
       <c r="E23" s="49"/>
       <c r="F23" s="49" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="G23" s="49"/>
       <c r="H23" s="49"/>
       <c r="I23" s="49" t="s">
-        <v>381</v>
+        <v>447</v>
       </c>
       <c r="J23" s="49"/>
       <c r="K23" s="49"/>
       <c r="L23" s="49"/>
       <c r="M23" s="49"/>
       <c r="N23" s="50" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="P23" s="21"/>
       <c r="Q23" s="21"/>
       <c r="T23" s="21"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C24" s="61" t="s">
-        <v>374</v>
-      </c>
-      <c r="D24" s="62"/>
-      <c r="E24" s="63"/>
-      <c r="F24" s="64">
+      <c r="C24" s="68" t="s">
+        <v>365</v>
+      </c>
+      <c r="D24" s="69"/>
+      <c r="E24" s="70"/>
+      <c r="F24" s="65">
         <f>0.048/0.581</f>
         <v>8.2616179001721177E-2</v>
       </c>
-      <c r="G24" s="65"/>
-      <c r="H24" s="66"/>
-      <c r="I24" s="58">
+      <c r="G24" s="66"/>
+      <c r="H24" s="67"/>
+      <c r="I24" s="71">
         <f>((T13+T15)/2)</f>
         <v>23.414850000000001</v>
       </c>
-      <c r="J24" s="59"/>
-      <c r="K24" s="59"/>
-      <c r="L24" s="59"/>
-      <c r="M24" s="60"/>
+      <c r="J24" s="72"/>
+      <c r="K24" s="72"/>
+      <c r="L24" s="72"/>
+      <c r="M24" s="73"/>
       <c r="N24" s="51">
         <f>((W13+W15)/2)</f>
         <v>2.2407199119595664E-4</v>
@@ -8166,25 +8159,25 @@
       <c r="T24" s="21"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C25" s="61" t="s">
-        <v>375</v>
-      </c>
-      <c r="D25" s="62"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="64">
+      <c r="C25" s="68" t="s">
+        <v>366</v>
+      </c>
+      <c r="D25" s="69"/>
+      <c r="E25" s="70"/>
+      <c r="F25" s="65">
         <f>0.104/0.581</f>
         <v>0.17900172117039587</v>
       </c>
-      <c r="G25" s="65"/>
-      <c r="H25" s="66"/>
-      <c r="I25" s="58">
+      <c r="G25" s="66"/>
+      <c r="H25" s="67"/>
+      <c r="I25" s="71">
         <f>T14</f>
         <v>97.18877280000001</v>
       </c>
-      <c r="J25" s="59"/>
-      <c r="K25" s="59"/>
-      <c r="L25" s="59"/>
-      <c r="M25" s="60"/>
+      <c r="J25" s="72"/>
+      <c r="K25" s="72"/>
+      <c r="L25" s="72"/>
+      <c r="M25" s="73"/>
       <c r="N25" s="51">
         <f>W14</f>
         <v>3.3521233224690123E-5</v>
@@ -8194,25 +8187,25 @@
       <c r="T25" s="21"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C26" s="61" t="s">
-        <v>373</v>
-      </c>
-      <c r="D26" s="62"/>
-      <c r="E26" s="63"/>
-      <c r="F26" s="64">
+      <c r="C26" s="68" t="s">
+        <v>364</v>
+      </c>
+      <c r="D26" s="69"/>
+      <c r="E26" s="70"/>
+      <c r="F26" s="65">
         <f>0.127/0.581</f>
         <v>0.21858864027538727</v>
       </c>
-      <c r="G26" s="65"/>
-      <c r="H26" s="66"/>
-      <c r="I26" s="58">
+      <c r="G26" s="66"/>
+      <c r="H26" s="67"/>
+      <c r="I26" s="71">
         <f>T16</f>
         <v>319.17554000000001</v>
       </c>
-      <c r="J26" s="59"/>
-      <c r="K26" s="59"/>
-      <c r="L26" s="59"/>
-      <c r="M26" s="60"/>
+      <c r="J26" s="72"/>
+      <c r="K26" s="72"/>
+      <c r="L26" s="72"/>
+      <c r="M26" s="73"/>
       <c r="N26" s="51">
         <f>W16</f>
         <v>1.1301491868138288E-5</v>
@@ -8222,25 +8215,25 @@
       <c r="T26" s="21"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C27" s="61" t="s">
-        <v>372</v>
-      </c>
-      <c r="D27" s="62"/>
-      <c r="E27" s="63"/>
-      <c r="F27" s="64">
+      <c r="C27" s="68" t="s">
+        <v>363</v>
+      </c>
+      <c r="D27" s="69"/>
+      <c r="E27" s="70"/>
+      <c r="F27" s="65">
         <f>0.144/0.581</f>
         <v>0.24784853700516352</v>
       </c>
-      <c r="G27" s="65"/>
-      <c r="H27" s="66"/>
-      <c r="I27" s="58">
+      <c r="G27" s="66"/>
+      <c r="H27" s="67"/>
+      <c r="I27" s="71">
         <f>((T10+T18)/2)</f>
         <v>1214.1039020000001</v>
       </c>
-      <c r="J27" s="59"/>
-      <c r="K27" s="59"/>
-      <c r="L27" s="59"/>
-      <c r="M27" s="60"/>
+      <c r="J27" s="72"/>
+      <c r="K27" s="72"/>
+      <c r="L27" s="72"/>
+      <c r="M27" s="73"/>
       <c r="N27" s="51">
         <f>((W10+W18)/2)</f>
         <v>5.481183696812177E-6</v>
@@ -8250,25 +8243,25 @@
       <c r="T27" s="21"/>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="C28" s="61" t="s">
-        <v>376</v>
-      </c>
-      <c r="D28" s="62"/>
-      <c r="E28" s="63"/>
-      <c r="F28" s="64">
+      <c r="C28" s="68" t="s">
+        <v>367</v>
+      </c>
+      <c r="D28" s="69"/>
+      <c r="E28" s="70"/>
+      <c r="F28" s="65">
         <f>0.157/0.581</f>
         <v>0.27022375215146299</v>
       </c>
-      <c r="G28" s="65"/>
-      <c r="H28" s="66"/>
-      <c r="I28" s="58">
+      <c r="G28" s="66"/>
+      <c r="H28" s="67"/>
+      <c r="I28" s="71">
         <f>((T9+T11+T12+T17+T19)/5)</f>
         <v>49678.416604960003</v>
       </c>
-      <c r="J28" s="59"/>
-      <c r="K28" s="59"/>
-      <c r="L28" s="59"/>
-      <c r="M28" s="60"/>
+      <c r="J28" s="72"/>
+      <c r="K28" s="72"/>
+      <c r="L28" s="72"/>
+      <c r="M28" s="73"/>
       <c r="N28" s="51">
         <f>((W9+W11+W12+W17+W19)/5)</f>
         <v>4.8514850079979492E-6</v>
@@ -8287,116 +8280,116 @@
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="G32" s="1" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="U32" s="9"/>
       <c r="W32" s="9"/>
     </row>
     <row r="33" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="D33" s="21">
         <v>502</v>
       </c>
       <c r="E33" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="T33" s="9"/>
     </row>
     <row r="34" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="D34" s="21">
         <v>250</v>
       </c>
       <c r="E34" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="T34" s="9"/>
     </row>
     <row r="35" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="D35" s="21">
         <f>D34/1.341</f>
         <v>186.42803877703207</v>
       </c>
       <c r="E35" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="36" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="D36" s="21">
         <v>2080</v>
       </c>
       <c r="E36" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="I36" s="8"/>
     </row>
     <row r="37" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>19</v>
+        <v>445</v>
       </c>
       <c r="D37" s="21">
         <f>D35*0.003412*D36</f>
         <v>1323.0723340790455</v>
       </c>
       <c r="E37" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
     </row>
     <row r="38" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D38" s="12">
         <f>(D33*D35)/(D37*10^6)</f>
         <v>7.0734511678239686E-5</v>
       </c>
       <c r="E38" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="I24:M24"/>
+    <mergeCell ref="I25:M25"/>
+    <mergeCell ref="I26:M26"/>
+    <mergeCell ref="I27:M27"/>
+    <mergeCell ref="I28:M28"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C28:E28"/>
     <mergeCell ref="F24:H24"/>
     <mergeCell ref="F25:H25"/>
     <mergeCell ref="F26:H26"/>
     <mergeCell ref="F27:H27"/>
     <mergeCell ref="F28:H28"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="I24:M24"/>
-    <mergeCell ref="I25:M25"/>
-    <mergeCell ref="I26:M26"/>
-    <mergeCell ref="I27:M27"/>
-    <mergeCell ref="I28:M28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G33" r:id="rId1" xr:uid="{89D540DE-65F8-419E-8E02-FD08F0D4350B}"/>
@@ -8419,7 +8412,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -8430,12 +8423,12 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="24" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -8443,94 +8436,94 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G5" s="1"/>
       <c r="K5" s="1"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D6">
         <f>AVERAGE(760,1000)</f>
         <v>880</v>
       </c>
       <c r="E6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D7">
         <f>AVERAGE(373.1,597)</f>
         <v>485.05</v>
       </c>
       <c r="E7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D11">
         <f>AVERAGE(975,1200)</f>
         <v>1087.5</v>
       </c>
       <c r="E11" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D12">
         <f>AVERAGE(1492.5,2238.8)</f>
         <v>1865.65</v>
       </c>
       <c r="E12" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D15">
         <v>1.5</v>
       </c>
       <c r="E15" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D16">
         <v>70</v>
       </c>
       <c r="E16" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="G18">
         <f>(D6)*(1.5*1000000)</f>
@@ -8539,7 +8532,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>156</v>
+        <v>448</v>
       </c>
       <c r="G19">
         <f>(1.5*1000000)*(0.7*8760)</f>
@@ -8548,7 +8541,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>157</v>
+        <v>449</v>
       </c>
       <c r="G20">
         <f>G19*3412</f>
@@ -8557,7 +8550,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="G21">
         <f>G18/G20</f>
@@ -8566,7 +8559,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="G22">
         <f>(D7*(1.5*1000000))/G20</f>
@@ -8575,7 +8568,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="G24">
         <f>(D11)*(1.5*1000000)</f>
@@ -8584,7 +8577,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>156</v>
+        <v>448</v>
       </c>
       <c r="G25">
         <f>(1.5*1000000)*(0.7*8760)</f>
@@ -8593,7 +8586,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>157</v>
+        <v>449</v>
       </c>
       <c r="G26">
         <f>G25*3412</f>
@@ -8602,7 +8595,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="G27">
         <f>G24/G26</f>
@@ -8611,7 +8604,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="G28">
         <f>(D12*(1.5*1000000))/G26</f>
@@ -8620,12 +8613,12 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="G32" s="12">
         <f>(G21*0.75)+(G27*0.25)</f>
@@ -8634,7 +8627,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="G33" s="9">
         <f>G32*0.6</f>
@@ -8646,7 +8639,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="G35" s="9">
         <f>(G22*0.75)+(G28*0.25)</f>
@@ -8671,7 +8664,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -8683,184 +8676,184 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="E3" s="39">
         <f>2758*1.03</f>
         <v>2840.7400000000002</v>
       </c>
       <c r="F3" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="H3" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>260</v>
+        <v>450</v>
       </c>
       <c r="E4">
         <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E5">
         <f>18*365</f>
         <v>6570</v>
       </c>
       <c r="F5" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="H5" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>181</v>
+        <v>443</v>
       </c>
       <c r="E7">
         <f>E4*E5</f>
         <v>118260</v>
       </c>
       <c r="F7" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>180</v>
+        <v>444</v>
       </c>
       <c r="E8">
         <f>E7*0.003412</f>
         <v>403.50312000000002</v>
       </c>
       <c r="F8" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="E9" s="12">
         <f>E3/(E8*10^6)</f>
         <v>7.0401933942914745E-6</v>
       </c>
       <c r="F9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="18"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="B16" s="8">
         <v>862500</v>
       </c>
       <c r="C16" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="B17" s="8">
         <v>1500000</v>
       </c>
       <c r="C17" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="B18" s="8">
         <f>AVERAGE(B16,B17)</f>
         <v>1181250</v>
       </c>
       <c r="C18" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B20" s="32">
         <v>8760</v>
       </c>
       <c r="C20" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B21" s="32">
         <v>6051100</v>
       </c>
       <c r="C21" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="B23">
         <f>B20*B21</f>
         <v>53007636000</v>
       </c>
       <c r="C23" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B24" s="12">
         <f>B18/B23</f>
         <v>2.2284525195577483E-5</v>
       </c>
       <c r="C24" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -8876,6 +8869,7 @@
   <dimension ref="A1:P83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
     <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
@@ -8886,7 +8880,7 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="B1" s="52"/>
       <c r="C1" s="52"/>
@@ -8909,7 +8903,7 @@
         <v>0.57060049240377109</v>
       </c>
       <c r="B2" t="s">
-        <v>421</v>
+        <v>411</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -8918,7 +8912,7 @@
         <v>266.66666666666669</v>
       </c>
       <c r="B3" t="s">
-        <v>425</v>
+        <v>415</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -8930,7 +8924,7 @@
         <v>8.2719018162705823E-4</v>
       </c>
       <c r="B5" t="s">
-        <v>431</v>
+        <v>421</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -8939,7 +8933,7 @@
         <v>3.1381977460259781E-3</v>
       </c>
       <c r="B6" t="s">
-        <v>432</v>
+        <v>422</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -8947,44 +8941,44 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C28" t="s">
-        <v>392</v>
+        <v>382</v>
       </c>
       <c r="D28" t="s">
-        <v>394</v>
+        <v>384</v>
       </c>
       <c r="E28" t="s">
-        <v>395</v>
+        <v>385</v>
       </c>
       <c r="F28" t="s">
-        <v>396</v>
+        <v>386</v>
       </c>
       <c r="G28" t="s">
-        <v>397</v>
+        <v>387</v>
       </c>
       <c r="H28" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
       <c r="I28" t="s">
-        <v>419</v>
+        <v>409</v>
       </c>
       <c r="M28" t="s">
-        <v>423</v>
+        <v>413</v>
       </c>
       <c r="N28" t="s">
-        <v>424</v>
+        <v>414</v>
       </c>
       <c r="O28" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="C29">
         <v>17000</v>
@@ -9007,7 +9001,7 @@
         <v>250</v>
       </c>
       <c r="L29" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="M29">
         <f>AVERAGE(C29:C31)*About!A149</f>
@@ -9024,7 +9018,7 @@
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C30">
         <v>17000</v>
@@ -9047,7 +9041,7 @@
         <v>250</v>
       </c>
       <c r="L30" t="s">
-        <v>422</v>
+        <v>412</v>
       </c>
       <c r="M30">
         <f>C32*About!A149</f>
@@ -9064,7 +9058,7 @@
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
       <c r="C31">
         <v>50000</v>
@@ -9089,7 +9083,7 @@
     </row>
     <row r="32" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>393</v>
+        <v>383</v>
       </c>
       <c r="C32">
         <v>55000</v>
@@ -9124,32 +9118,32 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="24" t="s">
-        <v>402</v>
+        <v>392</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
       <c r="D38" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="E38" t="s">
+        <v>408</v>
+      </c>
+      <c r="F38" t="s">
+        <v>416</v>
+      </c>
+      <c r="G38" t="s">
         <v>418</v>
       </c>
-      <c r="F38" t="s">
-        <v>426</v>
-      </c>
-      <c r="G38" t="s">
-        <v>428</v>
-      </c>
       <c r="H38" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>404</v>
+        <v>394</v>
       </c>
       <c r="C39">
         <v>2940</v>
@@ -9176,7 +9170,7 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
       <c r="C40">
         <v>113</v>
@@ -9203,33 +9197,33 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="F41" t="s">
-        <v>427</v>
+        <v>417</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="24" t="s">
-        <v>406</v>
+        <v>396</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C54" t="s">
-        <v>409</v>
+        <v>399</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>407</v>
+        <v>397</v>
       </c>
       <c r="C55" s="19">
         <v>0.54</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>417</v>
+        <v>407</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="C56" s="19">
         <v>0.52</v>
@@ -9240,32 +9234,32 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="24" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
     </row>
     <row r="81" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C81" t="s">
-        <v>413</v>
-      </c>
-      <c r="D81" t="s">
-        <v>414</v>
-      </c>
-      <c r="E81" t="s">
-        <v>415</v>
-      </c>
-      <c r="F81" t="s">
-        <v>416</v>
-      </c>
-      <c r="G81" t="s">
-        <v>430</v>
-      </c>
-      <c r="H81" t="s">
-        <v>128</v>
+      <c r="C81" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="E81" s="7" t="s">
+        <v>405</v>
+      </c>
+      <c r="F81" s="7" t="s">
+        <v>406</v>
+      </c>
+      <c r="G81" s="7" t="s">
+        <v>420</v>
+      </c>
+      <c r="H81" s="7" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="82" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B82" t="s">
-        <v>411</v>
+      <c r="B82" s="1" t="s">
+        <v>401</v>
       </c>
       <c r="C82">
         <v>28398</v>
@@ -9283,8 +9277,8 @@
       </c>
     </row>
     <row r="83" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B83" t="s">
-        <v>412</v>
+      <c r="B83" s="1" t="s">
+        <v>402</v>
       </c>
       <c r="C83">
         <v>25345</v>
@@ -9307,7 +9301,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>